<commit_message>
rescore the module arm against the regenerated eigengenes
</commit_message>
<xml_diff>
--- a/04_Figures/F04_association/c_data/results.xlsx
+++ b/04_Figures/F04_association/c_data/results.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="72">
   <si>
     <t xml:space="preserve">level</t>
   </si>
@@ -141,22 +141,7 @@
     <t xml:space="preserve">GOSLIM_DIGESTION</t>
   </si>
   <si>
-    <t xml:space="preserve">ME_green</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ME_salmon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ME_salmon@T2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ME_blue@T3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ME_green@T3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ME_tan@T3</t>
+    <t xml:space="preserve">ME_blue</t>
   </si>
   <si>
     <t xml:space="preserve">ACSL3</t>
@@ -165,7 +150,7 @@
     <t xml:space="preserve">GOSLIM_AMINO_ACID_METABOLIC_PROCESS</t>
   </si>
   <si>
-    <t xml:space="preserve">ME_green@T2</t>
+    <t xml:space="preserve">ME_red</t>
   </si>
   <si>
     <t xml:space="preserve">HALLMARK_KRAS_SIGNALING_UP</t>
@@ -192,16 +177,16 @@
     <t xml:space="preserve">HALLMARK_UNFOLDED_PROTEIN_RESPONSE</t>
   </si>
   <si>
-    <t xml:space="preserve">ME_blue</t>
+    <t xml:space="preserve">ME_black</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ME_brown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ME_green</t>
   </si>
   <si>
     <t xml:space="preserve">ME_greenyellow</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ME_red</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ME_tan</t>
   </si>
   <si>
     <t xml:space="preserve">RPL17</t>
@@ -216,10 +201,19 @@
     <t xml:space="preserve">HALLMARK_UNFOLDED_PROTEIN_RESPONSE@T3</t>
   </si>
   <si>
-    <t xml:space="preserve">ME_greenyellow@T3</t>
+    <t xml:space="preserve">ME_blue@T2</t>
   </si>
   <si>
-    <t xml:space="preserve">ME_red@T3</t>
+    <t xml:space="preserve">ME_black@T3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ME_brown@T3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ME_green@T3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ME_greenyellow@T3</t>
   </si>
   <si>
     <t xml:space="preserve">PGLS@T2</t>
@@ -603,7 +597,7 @@
         <v>11</v>
       </c>
       <c r="E2" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -612,7 +606,7 @@
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>0.00290840880033159</v>
+        <v>0.00262746819273299</v>
       </c>
     </row>
     <row r="3">
@@ -629,16 +623,16 @@
         <v>12</v>
       </c>
       <c r="E3" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0050027058155605</v>
+        <v>0.00544754815708406</v>
       </c>
     </row>
     <row r="4">
@@ -655,16 +649,16 @@
         <v>13</v>
       </c>
       <c r="E4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>0.00110612261301509</v>
+        <v>0.0011252670458588</v>
       </c>
     </row>
     <row r="5">
@@ -681,7 +675,7 @@
         <v>14</v>
       </c>
       <c r="E5" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -690,7 +684,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>0.000017230061084906</v>
+        <v>0.000012169796241576</v>
       </c>
     </row>
     <row r="6">
@@ -707,7 +701,7 @@
         <v>15</v>
       </c>
       <c r="E6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
@@ -716,7 +710,7 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>0.0000253219863875154</v>
+        <v>0.0000197825844385406</v>
       </c>
     </row>
     <row r="7">
@@ -733,7 +727,7 @@
         <v>16</v>
       </c>
       <c r="E7" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -742,7 +736,7 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0142707921642979</v>
+        <v>0.0150993555873671</v>
       </c>
     </row>
     <row r="8">
@@ -759,7 +753,7 @@
         <v>17</v>
       </c>
       <c r="E8" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
@@ -768,7 +762,7 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>0.0508877563674896</v>
+        <v>0.0430462035637821</v>
       </c>
     </row>
     <row r="9">
@@ -785,7 +779,7 @@
         <v>11</v>
       </c>
       <c r="E9" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
@@ -794,7 +788,7 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>8.64625200269644</v>
+        <v>7.47134685496238</v>
       </c>
     </row>
     <row r="10">
@@ -811,7 +805,7 @@
         <v>12</v>
       </c>
       <c r="E10" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F10" t="n">
         <v>2</v>
@@ -820,7 +814,7 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>11.6564593979345</v>
+        <v>11.2438997086154</v>
       </c>
     </row>
     <row r="11">
@@ -837,7 +831,7 @@
         <v>13</v>
       </c>
       <c r="E11" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
@@ -846,7 +840,7 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>49.1984273336599</v>
+        <v>49.5679068572702</v>
       </c>
     </row>
     <row r="12">
@@ -863,7 +857,7 @@
         <v>14</v>
       </c>
       <c r="E12" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
@@ -872,7 +866,7 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>2128.27249240115</v>
+        <v>1046.10887674005</v>
       </c>
     </row>
     <row r="13">
@@ -889,7 +883,7 @@
         <v>15</v>
       </c>
       <c r="E13" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
@@ -898,7 +892,7 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>2228.65335542619</v>
+        <v>1556.84903954256</v>
       </c>
     </row>
     <row r="14">
@@ -915,7 +909,7 @@
         <v>16</v>
       </c>
       <c r="E14" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
@@ -924,7 +918,7 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>3.25652010388715</v>
+        <v>2.93574629520819</v>
       </c>
     </row>
     <row r="15">
@@ -941,10 +935,10 @@
         <v>11</v>
       </c>
       <c r="E15" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
@@ -967,16 +961,16 @@
         <v>12</v>
       </c>
       <c r="E16" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F16" t="n">
         <v>2</v>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H16" t="n">
-        <v>0.262115173289534</v>
+        <v>0.244493985169229</v>
       </c>
     </row>
     <row r="17">
@@ -993,7 +987,7 @@
         <v>13</v>
       </c>
       <c r="E17" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
@@ -1002,7 +996,7 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>0.243729164129102</v>
+        <v>0.279571688265735</v>
       </c>
     </row>
     <row r="18">
@@ -1019,7 +1013,7 @@
         <v>14</v>
       </c>
       <c r="E18" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
@@ -1045,16 +1039,16 @@
         <v>15</v>
       </c>
       <c r="E19" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>0.203571428571429</v>
+        <v>0.171428571428571</v>
       </c>
     </row>
     <row r="20">
@@ -1071,16 +1065,16 @@
         <v>16</v>
       </c>
       <c r="E20" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>0.210714285714286</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="21">
@@ -1097,7 +1091,7 @@
         <v>17</v>
       </c>
       <c r="E21" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
@@ -1106,7 +1100,7 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>0.0523393298362787</v>
+        <v>0.042108848674314</v>
       </c>
     </row>
     <row r="22">
@@ -1123,7 +1117,7 @@
         <v>11</v>
       </c>
       <c r="E22" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F22" t="n">
         <v>0</v>
@@ -1132,7 +1126,7 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>0.00206205915241097</v>
+        <v>0.00203979642127084</v>
       </c>
     </row>
     <row r="23">
@@ -1149,16 +1143,16 @@
         <v>12</v>
       </c>
       <c r="E23" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G23" t="n">
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>0.00434924038756749</v>
+        <v>0.00446973025500284</v>
       </c>
     </row>
     <row r="24">
@@ -1175,16 +1169,16 @@
         <v>13</v>
       </c>
       <c r="E24" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>0.00113375938244125</v>
+        <v>0.00101034422976069</v>
       </c>
     </row>
     <row r="25">
@@ -1201,7 +1195,7 @@
         <v>14</v>
       </c>
       <c r="E25" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F25" t="n">
         <v>0</v>
@@ -1210,7 +1204,7 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>0.0000246225407425614</v>
+        <v>0.0000256561625278057</v>
       </c>
     </row>
     <row r="26">
@@ -1227,7 +1221,7 @@
         <v>15</v>
       </c>
       <c r="E26" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F26" t="n">
         <v>0</v>
@@ -1236,7 +1230,7 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>0.0000249713720573318</v>
+        <v>0.00002353149793292</v>
       </c>
     </row>
     <row r="27">
@@ -1253,16 +1247,16 @@
         <v>16</v>
       </c>
       <c r="E27" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F27" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H27" t="n">
-        <v>0.0261500728190795</v>
+        <v>0.0230729182193341</v>
       </c>
     </row>
     <row r="28">
@@ -1279,7 +1273,7 @@
         <v>17</v>
       </c>
       <c r="E28" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F28" t="n">
         <v>0</v>
@@ -1288,7 +1282,7 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>0.0410155765659239</v>
+        <v>0.0486298409445242</v>
       </c>
     </row>
     <row r="29">
@@ -1305,7 +1299,7 @@
         <v>11</v>
       </c>
       <c r="E29" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F29" t="n">
         <v>0</v>
@@ -1314,7 +1308,7 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>7.48592302124221</v>
+        <v>11.943645077654</v>
       </c>
     </row>
     <row r="30">
@@ -1331,16 +1325,16 @@
         <v>12</v>
       </c>
       <c r="E30" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G30" t="n">
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>10.6879984968909</v>
+        <v>15.5240312001011</v>
       </c>
     </row>
     <row r="31">
@@ -1357,16 +1351,16 @@
         <v>13</v>
       </c>
       <c r="E31" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G31" t="n">
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>53.2005089687761</v>
+        <v>84.4532272987479</v>
       </c>
     </row>
     <row r="32">
@@ -1383,7 +1377,7 @@
         <v>14</v>
       </c>
       <c r="E32" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F32" t="n">
         <v>0</v>
@@ -1392,7 +1386,7 @@
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>3001.11423376834</v>
+        <v>2989.53923859455</v>
       </c>
     </row>
     <row r="33">
@@ -1409,7 +1403,7 @@
         <v>15</v>
       </c>
       <c r="E33" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F33" t="n">
         <v>0</v>
@@ -1418,7 +1412,7 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>2183.62020625647</v>
+        <v>2554.98110707804</v>
       </c>
     </row>
     <row r="34">
@@ -1435,16 +1429,16 @@
         <v>16</v>
       </c>
       <c r="E34" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F34" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G34" t="n">
         <v>1</v>
       </c>
       <c r="H34" t="n">
-        <v>5.26890555325019</v>
+        <v>5.11997141402431</v>
       </c>
     </row>
     <row r="35">
@@ -1461,7 +1455,7 @@
         <v>11</v>
       </c>
       <c r="E35" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F35" t="n">
         <v>0</v>
@@ -1470,7 +1464,7 @@
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>0.125</v>
+        <v>0.139285714285714</v>
       </c>
     </row>
     <row r="36">
@@ -1487,16 +1481,16 @@
         <v>12</v>
       </c>
       <c r="E36" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G36" t="n">
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>0.218062202988772</v>
+        <v>0.169603935657934</v>
       </c>
     </row>
     <row r="37">
@@ -1513,16 +1507,16 @@
         <v>13</v>
       </c>
       <c r="E37" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F37" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G37" t="n">
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>0.24394864113362</v>
+        <v>0.238567421108613</v>
       </c>
     </row>
     <row r="38">
@@ -1539,7 +1533,7 @@
         <v>14</v>
       </c>
       <c r="E38" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F38" t="n">
         <v>0</v>
@@ -1548,7 +1542,7 @@
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>0.178571428571429</v>
+        <v>0.196428571428571</v>
       </c>
     </row>
     <row r="39">
@@ -1565,7 +1559,7 @@
         <v>15</v>
       </c>
       <c r="E39" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F39" t="n">
         <v>0</v>
@@ -1574,7 +1568,7 @@
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>0.153571428571429</v>
+        <v>0.110714285714286</v>
       </c>
     </row>
     <row r="40">
@@ -1591,16 +1585,16 @@
         <v>16</v>
       </c>
       <c r="E40" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G40" t="n">
         <v>1</v>
       </c>
       <c r="H40" t="n">
-        <v>0.35</v>
+        <v>0.303571428571428</v>
       </c>
     </row>
     <row r="41">
@@ -1617,7 +1611,7 @@
         <v>17</v>
       </c>
       <c r="E41" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F41" t="n">
         <v>0</v>
@@ -1626,7 +1620,7 @@
         <v>0</v>
       </c>
       <c r="H41" t="n">
-        <v>0.0742406474776733</v>
+        <v>0.0566122472545513</v>
       </c>
     </row>
     <row r="42">
@@ -1643,16 +1637,16 @@
         <v>11</v>
       </c>
       <c r="E42" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F42" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G42" t="n">
         <v>0</v>
       </c>
       <c r="H42" t="n">
-        <v>0.00411803885045364</v>
+        <v>0.00469261581250222</v>
       </c>
     </row>
     <row r="43">
@@ -1669,7 +1663,7 @@
         <v>12</v>
       </c>
       <c r="E43" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F43" t="n">
         <v>0</v>
@@ -1678,7 +1672,7 @@
         <v>0</v>
       </c>
       <c r="H43" t="n">
-        <v>0.0023614443502669</v>
+        <v>0.00150313104441507</v>
       </c>
     </row>
     <row r="44">
@@ -1695,7 +1689,7 @@
         <v>13</v>
       </c>
       <c r="E44" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F44" t="n">
         <v>0</v>
@@ -1704,7 +1698,7 @@
         <v>0</v>
       </c>
       <c r="H44" t="n">
-        <v>0.000707332939178</v>
+        <v>0.000785484170594167</v>
       </c>
     </row>
     <row r="45">
@@ -1721,7 +1715,7 @@
         <v>14</v>
       </c>
       <c r="E45" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F45" t="n">
         <v>1</v>
@@ -1730,7 +1724,7 @@
         <v>0</v>
       </c>
       <c r="H45" t="n">
-        <v>0.0000196050136280696</v>
+        <v>0.0000162205768505554</v>
       </c>
     </row>
     <row r="46">
@@ -1747,7 +1741,7 @@
         <v>15</v>
       </c>
       <c r="E46" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F46" t="n">
         <v>1</v>
@@ -1756,7 +1750,7 @@
         <v>0</v>
       </c>
       <c r="H46" t="n">
-        <v>0.0000272103327405134</v>
+        <v>0.0000220220509735622</v>
       </c>
     </row>
     <row r="47">
@@ -1773,16 +1767,16 @@
         <v>16</v>
       </c>
       <c r="E47" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F47" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G47" t="n">
         <v>0</v>
       </c>
       <c r="H47" t="n">
-        <v>0.0189282140002292</v>
+        <v>0.0339578479680035</v>
       </c>
     </row>
     <row r="48">
@@ -1799,7 +1793,7 @@
         <v>17</v>
       </c>
       <c r="E48" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F48" t="n">
         <v>1</v>
@@ -1808,7 +1802,7 @@
         <v>0</v>
       </c>
       <c r="H48" t="n">
-        <v>0.0680405600197775</v>
+        <v>0.0807219342523098</v>
       </c>
     </row>
     <row r="49">
@@ -1825,7 +1819,7 @@
         <v>11</v>
       </c>
       <c r="E49" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F49" t="n">
         <v>3</v>
@@ -1834,7 +1828,7 @@
         <v>0</v>
       </c>
       <c r="H49" t="n">
-        <v>13.8942291743769</v>
+        <v>18.4204749635253</v>
       </c>
     </row>
     <row r="50">
@@ -1851,7 +1845,7 @@
         <v>12</v>
       </c>
       <c r="E50" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F50" t="n">
         <v>0</v>
@@ -1860,7 +1854,7 @@
         <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>4.41124334728713</v>
+        <v>4.17699711740554</v>
       </c>
     </row>
     <row r="51">
@@ -1877,7 +1871,7 @@
         <v>13</v>
       </c>
       <c r="E51" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F51" t="n">
         <v>0</v>
@@ -1886,7 +1880,7 @@
         <v>0</v>
       </c>
       <c r="H51" t="n">
-        <v>31.2322969350702</v>
+        <v>31.6953098820755</v>
       </c>
     </row>
     <row r="52">
@@ -1903,7 +1897,7 @@
         <v>14</v>
       </c>
       <c r="E52" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F52" t="n">
         <v>0</v>
@@ -1912,7 +1906,7 @@
         <v>0</v>
       </c>
       <c r="H52" t="n">
-        <v>1964.43828997944</v>
+        <v>1945.49333788651</v>
       </c>
     </row>
     <row r="53">
@@ -1929,7 +1923,7 @@
         <v>15</v>
       </c>
       <c r="E53" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F53" t="n">
         <v>0</v>
@@ -1938,7 +1932,7 @@
         <v>0</v>
       </c>
       <c r="H53" t="n">
-        <v>1644.84547012377</v>
+        <v>1872.48876751234</v>
       </c>
     </row>
     <row r="54">
@@ -1955,16 +1949,16 @@
         <v>16</v>
       </c>
       <c r="E54" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F54" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G54" t="n">
         <v>0</v>
       </c>
       <c r="H54" t="n">
-        <v>4.41347363758293</v>
+        <v>5.50187255817476</v>
       </c>
     </row>
     <row r="55">
@@ -1981,7 +1975,7 @@
         <v>11</v>
       </c>
       <c r="E55" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F55" t="n">
         <v>2</v>
@@ -1990,7 +1984,7 @@
         <v>0</v>
       </c>
       <c r="H55" t="n">
-        <v>0.260714285714286</v>
+        <v>0.217857142857143</v>
       </c>
     </row>
     <row r="56">
@@ -2007,7 +2001,7 @@
         <v>12</v>
       </c>
       <c r="E56" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F56" t="n">
         <v>0</v>
@@ -2016,7 +2010,7 @@
         <v>0</v>
       </c>
       <c r="H56" t="n">
-        <v>0.110132425751905</v>
+        <v>0.132158910902286</v>
       </c>
     </row>
     <row r="57">
@@ -2033,7 +2027,7 @@
         <v>13</v>
       </c>
       <c r="E57" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F57" t="n">
         <v>0</v>
@@ -2059,10 +2053,10 @@
         <v>14</v>
       </c>
       <c r="E58" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G58" t="n">
         <v>0</v>
@@ -2085,7 +2079,7 @@
         <v>15</v>
       </c>
       <c r="E59" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F59" t="n">
         <v>0</v>
@@ -2094,7 +2088,7 @@
         <v>0</v>
       </c>
       <c r="H59" t="n">
-        <v>0.192857142857143</v>
+        <v>0.157142857142857</v>
       </c>
     </row>
     <row r="60">
@@ -2111,7 +2105,7 @@
         <v>16</v>
       </c>
       <c r="E60" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F60" t="n">
         <v>4</v>
@@ -2120,7 +2114,7 @@
         <v>4</v>
       </c>
       <c r="H60" t="n">
-        <v>0.392857142857143</v>
+        <v>0.403571428571428</v>
       </c>
     </row>
     <row r="61">
@@ -2137,7 +2131,7 @@
         <v>17</v>
       </c>
       <c r="E61" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F61" t="n">
         <v>0</v>
@@ -2146,7 +2140,7 @@
         <v>0</v>
       </c>
       <c r="H61" t="n">
-        <v>0.0496455215776404</v>
+        <v>0.0606463650879815</v>
       </c>
     </row>
     <row r="62">
@@ -2163,7 +2157,7 @@
         <v>11</v>
       </c>
       <c r="E62" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F62" t="n">
         <v>2</v>
@@ -2172,7 +2166,7 @@
         <v>0</v>
       </c>
       <c r="H62" t="n">
-        <v>0.00758196482054729</v>
+        <v>0.00782933833598707</v>
       </c>
     </row>
     <row r="63">
@@ -2189,7 +2183,7 @@
         <v>12</v>
       </c>
       <c r="E63" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F63" t="n">
         <v>0</v>
@@ -2198,7 +2192,7 @@
         <v>0</v>
       </c>
       <c r="H63" t="n">
-        <v>0.00584028857138172</v>
+        <v>0.00457628131680316</v>
       </c>
     </row>
     <row r="64">
@@ -2215,7 +2209,7 @@
         <v>13</v>
       </c>
       <c r="E64" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F64" t="n">
         <v>0</v>
@@ -2224,7 +2218,7 @@
         <v>0</v>
       </c>
       <c r="H64" t="n">
-        <v>0.0012598429492778</v>
+        <v>0.00120709932049167</v>
       </c>
     </row>
     <row r="65">
@@ -2241,7 +2235,7 @@
         <v>14</v>
       </c>
       <c r="E65" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F65" t="n">
         <v>0</v>
@@ -2250,7 +2244,7 @@
         <v>0</v>
       </c>
       <c r="H65" t="n">
-        <v>0.0000276351002658943</v>
+        <v>0.0000247401769014283</v>
       </c>
     </row>
     <row r="66">
@@ -2267,7 +2261,7 @@
         <v>15</v>
       </c>
       <c r="E66" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F66" t="n">
         <v>0</v>
@@ -2276,7 +2270,7 @@
         <v>0</v>
       </c>
       <c r="H66" t="n">
-        <v>0.0000312329498200107</v>
+        <v>0.0000320393038005807</v>
       </c>
     </row>
     <row r="67">
@@ -2293,16 +2287,16 @@
         <v>16</v>
       </c>
       <c r="E67" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F67" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G67" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H67" t="n">
-        <v>0.0204814290020186</v>
+        <v>0.0222154717487911</v>
       </c>
     </row>
     <row r="68">
@@ -2319,16 +2313,16 @@
         <v>17</v>
       </c>
       <c r="E68" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G68" t="n">
         <v>0</v>
       </c>
       <c r="H68" t="n">
-        <v>0.104203373089207</v>
+        <v>0.111306484229624</v>
       </c>
     </row>
     <row r="69">
@@ -2345,16 +2339,16 @@
         <v>11</v>
       </c>
       <c r="E69" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G69" t="n">
         <v>0</v>
       </c>
       <c r="H69" t="n">
-        <v>13.0627200078071</v>
+        <v>17.7718488826961</v>
       </c>
     </row>
     <row r="70">
@@ -2371,7 +2365,7 @@
         <v>12</v>
       </c>
       <c r="E70" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F70" t="n">
         <v>0</v>
@@ -2380,7 +2374,7 @@
         <v>0</v>
       </c>
       <c r="H70" t="n">
-        <v>8.10776723815438</v>
+        <v>5.82233929475659</v>
       </c>
     </row>
     <row r="71">
@@ -2397,7 +2391,7 @@
         <v>13</v>
       </c>
       <c r="E71" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F71" t="n">
         <v>0</v>
@@ -2406,7 +2400,7 @@
         <v>0</v>
       </c>
       <c r="H71" t="n">
-        <v>36.8458058819689</v>
+        <v>36.6676652375296</v>
       </c>
     </row>
     <row r="72">
@@ -2423,7 +2417,7 @@
         <v>14</v>
       </c>
       <c r="E72" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F72" t="n">
         <v>0</v>
@@ -2432,7 +2426,7 @@
         <v>0</v>
       </c>
       <c r="H72" t="n">
-        <v>1728.85729581191</v>
+        <v>1789.85514091352</v>
       </c>
     </row>
     <row r="73">
@@ -2449,7 +2443,7 @@
         <v>15</v>
       </c>
       <c r="E73" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F73" t="n">
         <v>0</v>
@@ -2458,7 +2452,7 @@
         <v>0</v>
       </c>
       <c r="H73" t="n">
-        <v>1553.89321443555</v>
+        <v>1620.70298921829</v>
       </c>
     </row>
     <row r="74">
@@ -2475,16 +2469,16 @@
         <v>16</v>
       </c>
       <c r="E74" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F74" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G74" t="n">
         <v>0</v>
       </c>
       <c r="H74" t="n">
-        <v>2.05296457953113</v>
+        <v>2.55496905702803</v>
       </c>
     </row>
     <row r="75">
@@ -2501,16 +2495,16 @@
         <v>11</v>
       </c>
       <c r="E75" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G75" t="n">
         <v>0</v>
       </c>
       <c r="H75" t="n">
-        <v>0.160714285714286</v>
+        <v>0.296428571428571</v>
       </c>
     </row>
     <row r="76">
@@ -2527,7 +2521,7 @@
         <v>12</v>
       </c>
       <c r="E76" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F76" t="n">
         <v>0</v>
@@ -2536,7 +2530,7 @@
         <v>0</v>
       </c>
       <c r="H76" t="n">
-        <v>0.264317821804572</v>
+        <v>0.202643663383505</v>
       </c>
     </row>
     <row r="77">
@@ -2553,7 +2547,7 @@
         <v>13</v>
       </c>
       <c r="E77" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F77" t="n">
         <v>0</v>
@@ -2562,7 +2556,7 @@
         <v>0</v>
       </c>
       <c r="H77" t="n">
-        <v>0.24394864113362</v>
+        <v>0.206280100958575</v>
       </c>
     </row>
     <row r="78">
@@ -2579,7 +2573,7 @@
         <v>14</v>
       </c>
       <c r="E78" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F78" t="n">
         <v>0</v>
@@ -2588,7 +2582,7 @@
         <v>0</v>
       </c>
       <c r="H78" t="n">
-        <v>0.167857142857143</v>
+        <v>0.171428571428571</v>
       </c>
     </row>
     <row r="79">
@@ -2605,7 +2599,7 @@
         <v>15</v>
       </c>
       <c r="E79" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F79" t="n">
         <v>0</v>
@@ -2614,7 +2608,7 @@
         <v>0</v>
       </c>
       <c r="H79" t="n">
-        <v>0.207142857142857</v>
+        <v>0.221428571428571</v>
       </c>
     </row>
     <row r="80">
@@ -2631,16 +2625,16 @@
         <v>16</v>
       </c>
       <c r="E80" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F80" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G80" t="n">
         <v>0</v>
       </c>
       <c r="H80" t="n">
-        <v>0.207142857142857</v>
+        <v>0.275</v>
       </c>
     </row>
     <row r="81">
@@ -2657,7 +2651,7 @@
         <v>17</v>
       </c>
       <c r="E81" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F81" t="n">
         <v>0</v>
@@ -2666,7 +2660,7 @@
         <v>0</v>
       </c>
       <c r="H81" t="n">
-        <v>0.0851740904473904</v>
+        <v>0.116606289952657</v>
       </c>
     </row>
     <row r="82">
@@ -2683,7 +2677,7 @@
         <v>11</v>
       </c>
       <c r="E82" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F82" t="n">
         <v>0</v>
@@ -2692,7 +2686,7 @@
         <v>0</v>
       </c>
       <c r="H82" t="n">
-        <v>0.00651074311506289</v>
+        <v>0.00583363322851157</v>
       </c>
     </row>
     <row r="83">
@@ -2709,7 +2703,7 @@
         <v>12</v>
       </c>
       <c r="E83" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F83" t="n">
         <v>0</v>
@@ -2718,7 +2712,7 @@
         <v>0</v>
       </c>
       <c r="H83" t="n">
-        <v>0.00878184776028905</v>
+        <v>0.00725086831226831</v>
       </c>
     </row>
     <row r="84">
@@ -2735,7 +2729,7 @@
         <v>13</v>
       </c>
       <c r="E84" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F84" t="n">
         <v>0</v>
@@ -2744,7 +2738,7 @@
         <v>0</v>
       </c>
       <c r="H84" t="n">
-        <v>0.000629041978578544</v>
+        <v>0.00101405007158605</v>
       </c>
     </row>
     <row r="85">
@@ -2761,7 +2755,7 @@
         <v>14</v>
       </c>
       <c r="E85" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F85" t="n">
         <v>0</v>
@@ -2770,7 +2764,7 @@
         <v>0</v>
       </c>
       <c r="H85" t="n">
-        <v>0.0000135365918507659</v>
+        <v>0.0000132591822845853</v>
       </c>
     </row>
     <row r="86">
@@ -2787,7 +2781,7 @@
         <v>15</v>
       </c>
       <c r="E86" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F86" t="n">
         <v>0</v>
@@ -2796,7 +2790,7 @@
         <v>0</v>
       </c>
       <c r="H86" t="n">
-        <v>0.000019403648592854</v>
+        <v>0.0000217062016168289</v>
       </c>
     </row>
     <row r="87">
@@ -2813,7 +2807,7 @@
         <v>16</v>
       </c>
       <c r="E87" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F87" t="n">
         <v>1</v>
@@ -2822,7 +2816,7 @@
         <v>0</v>
       </c>
       <c r="H87" t="n">
-        <v>0.0177960018151424</v>
+        <v>0.0168351774117431</v>
       </c>
     </row>
     <row r="88">
@@ -2839,7 +2833,7 @@
         <v>17</v>
       </c>
       <c r="E88" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F88" t="n">
         <v>0</v>
@@ -2848,7 +2842,7 @@
         <v>0</v>
       </c>
       <c r="H88" t="n">
-        <v>0.0384367287846884</v>
+        <v>0.0239887874837593</v>
       </c>
     </row>
     <row r="89">
@@ -2865,7 +2859,7 @@
         <v>11</v>
       </c>
       <c r="E89" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F89" t="n">
         <v>0</v>
@@ -2874,7 +2868,7 @@
         <v>0</v>
       </c>
       <c r="H89" t="n">
-        <v>7.27273150518333</v>
+        <v>7.3987360821477</v>
       </c>
     </row>
     <row r="90">
@@ -2891,7 +2885,7 @@
         <v>12</v>
       </c>
       <c r="E90" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F90" t="n">
         <v>0</v>
@@ -2900,7 +2894,7 @@
         <v>0</v>
       </c>
       <c r="H90" t="n">
-        <v>6.32355935926166</v>
+        <v>6.79739740142915</v>
       </c>
     </row>
     <row r="91">
@@ -2917,7 +2911,7 @@
         <v>13</v>
       </c>
       <c r="E91" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F91" t="n">
         <v>0</v>
@@ -2926,7 +2920,7 @@
         <v>0</v>
       </c>
       <c r="H91" t="n">
-        <v>20.327775943847</v>
+        <v>22.8383509793066</v>
       </c>
     </row>
     <row r="92">
@@ -2943,7 +2937,7 @@
         <v>14</v>
       </c>
       <c r="E92" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F92" t="n">
         <v>0</v>
@@ -2952,7 +2946,7 @@
         <v>0</v>
       </c>
       <c r="H92" t="n">
-        <v>721.844859689035</v>
+        <v>711.914004079463</v>
       </c>
     </row>
     <row r="93">
@@ -2969,7 +2963,7 @@
         <v>15</v>
       </c>
       <c r="E93" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F93" t="n">
         <v>0</v>
@@ -2978,7 +2972,7 @@
         <v>0</v>
       </c>
       <c r="H93" t="n">
-        <v>1124.94073900446</v>
+        <v>884.539939422603</v>
       </c>
     </row>
     <row r="94">
@@ -2995,7 +2989,7 @@
         <v>16</v>
       </c>
       <c r="E94" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F94" t="n">
         <v>1</v>
@@ -3004,7 +2998,7 @@
         <v>0</v>
       </c>
       <c r="H94" t="n">
-        <v>1.92158555780889</v>
+        <v>1.52728730003724</v>
       </c>
     </row>
     <row r="95">
@@ -3021,16 +3015,16 @@
         <v>11</v>
       </c>
       <c r="E95" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F95" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G95" t="n">
         <v>0</v>
       </c>
       <c r="H95" t="n">
-        <v>0.208791208791209</v>
+        <v>0.221978021978022</v>
       </c>
     </row>
     <row r="96">
@@ -3047,7 +3041,7 @@
         <v>12</v>
       </c>
       <c r="E96" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F96" t="n">
         <v>0</v>
@@ -3056,7 +3050,7 @@
         <v>0</v>
       </c>
       <c r="H96" t="n">
-        <v>0.225896173973403</v>
+        <v>0.209367185633885</v>
       </c>
     </row>
     <row r="97">
@@ -3073,7 +3067,7 @@
         <v>13</v>
       </c>
       <c r="E97" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F97" t="n">
         <v>0</v>
@@ -3082,7 +3076,7 @@
         <v>0</v>
       </c>
       <c r="H97" t="n">
-        <v>0.156734419398595</v>
+        <v>0.183224743803992</v>
       </c>
     </row>
     <row r="98">
@@ -3099,7 +3093,7 @@
         <v>14</v>
       </c>
       <c r="E98" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F98" t="n">
         <v>0</v>
@@ -3108,7 +3102,7 @@
         <v>0</v>
       </c>
       <c r="H98" t="n">
-        <v>0.103296703296703</v>
+        <v>0.0769230769230769</v>
       </c>
     </row>
     <row r="99">
@@ -3125,7 +3119,7 @@
         <v>15</v>
       </c>
       <c r="E99" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F99" t="n">
         <v>0</v>
@@ -3134,7 +3128,7 @@
         <v>0</v>
       </c>
       <c r="H99" t="n">
-        <v>0.164835164835165</v>
+        <v>0.156043956043956</v>
       </c>
     </row>
     <row r="100">
@@ -3151,7 +3145,7 @@
         <v>16</v>
       </c>
       <c r="E100" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F100" t="n">
         <v>1</v>
@@ -3160,7 +3154,7 @@
         <v>0</v>
       </c>
       <c r="H100" t="n">
-        <v>0.265934065934066</v>
+        <v>0.23956043956044</v>
       </c>
     </row>
     <row r="101">
@@ -3177,7 +3171,7 @@
         <v>17</v>
       </c>
       <c r="E101" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F101" t="n">
         <v>0</v>
@@ -3186,7 +3180,7 @@
         <v>0</v>
       </c>
       <c r="H101" t="n">
-        <v>0.0772201899729983</v>
+        <v>0.0779271400254632</v>
       </c>
     </row>
     <row r="102">
@@ -3203,7 +3197,7 @@
         <v>11</v>
       </c>
       <c r="E102" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F102" t="n">
         <v>0</v>
@@ -3212,7 +3206,7 @@
         <v>0</v>
       </c>
       <c r="H102" t="n">
-        <v>0.00248318340548715</v>
+        <v>0.00241133373013234</v>
       </c>
     </row>
     <row r="103">
@@ -3229,16 +3223,16 @@
         <v>12</v>
       </c>
       <c r="E103" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F103" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G103" t="n">
         <v>0</v>
       </c>
       <c r="H103" t="n">
-        <v>0.00680429725284685</v>
+        <v>0.0062365768162108</v>
       </c>
     </row>
     <row r="104">
@@ -3255,7 +3249,7 @@
         <v>13</v>
       </c>
       <c r="E104" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F104" t="n">
         <v>0</v>
@@ -3264,7 +3258,7 @@
         <v>0</v>
       </c>
       <c r="H104" t="n">
-        <v>0.00100455601498451</v>
+        <v>0.000780765751582357</v>
       </c>
     </row>
     <row r="105">
@@ -3281,7 +3275,7 @@
         <v>14</v>
       </c>
       <c r="E105" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F105" t="n">
         <v>0</v>
@@ -3290,7 +3284,7 @@
         <v>0</v>
       </c>
       <c r="H105" t="n">
-        <v>0.0000244469620012894</v>
+        <v>0.0000143230281940479</v>
       </c>
     </row>
     <row r="106">
@@ -3307,7 +3301,7 @@
         <v>15</v>
       </c>
       <c r="E106" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F106" t="n">
         <v>0</v>
@@ -3316,7 +3310,7 @@
         <v>0</v>
       </c>
       <c r="H106" t="n">
-        <v>0.0000283861026907639</v>
+        <v>0.0000166555417076123</v>
       </c>
     </row>
     <row r="107">
@@ -3333,16 +3327,16 @@
         <v>16</v>
       </c>
       <c r="E107" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F107" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G107" t="n">
         <v>0</v>
       </c>
       <c r="H107" t="n">
-        <v>0.0131266784915903</v>
+        <v>0.0150031270594946</v>
       </c>
     </row>
     <row r="108">
@@ -3359,7 +3353,7 @@
         <v>17</v>
       </c>
       <c r="E108" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F108" t="n">
         <v>0</v>
@@ -3368,7 +3362,7 @@
         <v>0</v>
       </c>
       <c r="H108" t="n">
-        <v>0.071586959091947</v>
+        <v>0.0930190516412853</v>
       </c>
     </row>
     <row r="109">
@@ -3385,7 +3379,7 @@
         <v>11</v>
       </c>
       <c r="E109" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F109" t="n">
         <v>0</v>
@@ -3394,7 +3388,7 @@
         <v>0</v>
       </c>
       <c r="H109" t="n">
-        <v>4.62351749580375</v>
+        <v>5.44004819871796</v>
       </c>
     </row>
     <row r="110">
@@ -3411,16 +3405,16 @@
         <v>12</v>
       </c>
       <c r="E110" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F110" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G110" t="n">
         <v>0</v>
       </c>
       <c r="H110" t="n">
-        <v>7.01211867705781</v>
+        <v>9.55869811208761</v>
       </c>
     </row>
     <row r="111">
@@ -3437,7 +3431,7 @@
         <v>13</v>
       </c>
       <c r="E111" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F111" t="n">
         <v>0</v>
@@ -3446,7 +3440,7 @@
         <v>0</v>
       </c>
       <c r="H111" t="n">
-        <v>40.5340840271943</v>
+        <v>35.1482371921958</v>
       </c>
     </row>
     <row r="112">
@@ -3463,16 +3457,16 @@
         <v>14</v>
       </c>
       <c r="E112" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F112" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G112" t="n">
         <v>0</v>
       </c>
       <c r="H112" t="n">
-        <v>1494.46784401706</v>
+        <v>1019.06929145149</v>
       </c>
     </row>
     <row r="113">
@@ -3489,7 +3483,7 @@
         <v>15</v>
       </c>
       <c r="E113" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F113" t="n">
         <v>0</v>
@@ -3498,7 +3492,7 @@
         <v>0</v>
       </c>
       <c r="H113" t="n">
-        <v>1388.78967438055</v>
+        <v>815.492404145446</v>
       </c>
     </row>
     <row r="114">
@@ -3515,7 +3509,7 @@
         <v>16</v>
       </c>
       <c r="E114" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F114" t="n">
         <v>1</v>
@@ -3524,7 +3518,7 @@
         <v>0</v>
       </c>
       <c r="H114" t="n">
-        <v>1.9749790766767</v>
+        <v>1.53714101238503</v>
       </c>
     </row>
     <row r="115">
@@ -3541,7 +3535,7 @@
         <v>11</v>
       </c>
       <c r="E115" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F115" t="n">
         <v>0</v>
@@ -3550,7 +3544,7 @@
         <v>0</v>
       </c>
       <c r="H115" t="n">
-        <v>0.125274725274725</v>
+        <v>0.0725274725274725</v>
       </c>
     </row>
     <row r="116">
@@ -3567,7 +3561,7 @@
         <v>12</v>
       </c>
       <c r="E116" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F116" t="n">
         <v>2</v>
@@ -3576,7 +3570,7 @@
         <v>0</v>
       </c>
       <c r="H116" t="n">
-        <v>0.236915499533081</v>
+        <v>0.256199319262518</v>
       </c>
     </row>
     <row r="117">
@@ -3593,7 +3587,7 @@
         <v>13</v>
       </c>
       <c r="E117" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F117" t="n">
         <v>0</v>
@@ -3602,7 +3596,7 @@
         <v>0</v>
       </c>
       <c r="H117" t="n">
-        <v>0.200884960074256</v>
+        <v>0.143489257195897</v>
       </c>
     </row>
     <row r="118">
@@ -3619,7 +3613,7 @@
         <v>14</v>
       </c>
       <c r="E118" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F118" t="n">
         <v>0</v>
@@ -3628,7 +3622,7 @@
         <v>0</v>
       </c>
       <c r="H118" t="n">
-        <v>0.138461538461538</v>
+        <v>0.134065934065934</v>
       </c>
     </row>
     <row r="119">
@@ -3645,7 +3639,7 @@
         <v>15</v>
       </c>
       <c r="E119" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F119" t="n">
         <v>0</v>
@@ -3654,7 +3648,7 @@
         <v>0</v>
       </c>
       <c r="H119" t="n">
-        <v>0.142857142857143</v>
+        <v>0.116483516483516</v>
       </c>
     </row>
     <row r="120">
@@ -3671,16 +3665,16 @@
         <v>16</v>
       </c>
       <c r="E120" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F120" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G120" t="n">
         <v>0</v>
       </c>
       <c r="H120" t="n">
-        <v>0.0637362637362637</v>
+        <v>0.0813186813186813</v>
       </c>
     </row>
     <row r="121">
@@ -3697,7 +3691,7 @@
         <v>17</v>
       </c>
       <c r="E121" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F121" t="n">
         <v>0</v>
@@ -3706,7 +3700,7 @@
         <v>0</v>
       </c>
       <c r="H121" t="n">
-        <v>0.051645108243261</v>
+        <v>0.0537246405350849</v>
       </c>
     </row>
     <row r="122">
@@ -3723,16 +3717,16 @@
         <v>11</v>
       </c>
       <c r="E122" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F122" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G122" t="n">
         <v>0</v>
       </c>
       <c r="H122" t="n">
-        <v>0.00247246904545623</v>
+        <v>0.00225963595743908</v>
       </c>
     </row>
     <row r="123">
@@ -3749,16 +3743,16 @@
         <v>12</v>
       </c>
       <c r="E123" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F123" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G123" t="n">
         <v>0</v>
       </c>
       <c r="H123" t="n">
-        <v>0.0049824353219826</v>
+        <v>0.00493375806251794</v>
       </c>
     </row>
     <row r="124">
@@ -3775,7 +3769,7 @@
         <v>13</v>
       </c>
       <c r="E124" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F124" t="n">
         <v>1</v>
@@ -3784,7 +3778,7 @@
         <v>0</v>
       </c>
       <c r="H124" t="n">
-        <v>0.000850308101323678</v>
+        <v>0.00100234676368229</v>
       </c>
     </row>
     <row r="125">
@@ -3801,7 +3795,7 @@
         <v>14</v>
       </c>
       <c r="E125" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F125" t="n">
         <v>1</v>
@@ -3810,7 +3804,7 @@
         <v>0</v>
       </c>
       <c r="H125" t="n">
-        <v>0.0000215579778367726</v>
+        <v>0.0000169781436644301</v>
       </c>
     </row>
     <row r="126">
@@ -3827,7 +3821,7 @@
         <v>15</v>
       </c>
       <c r="E126" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F126" t="n">
         <v>1</v>
@@ -3836,7 +3830,7 @@
         <v>0</v>
       </c>
       <c r="H126" t="n">
-        <v>0.0000233844497863228</v>
+        <v>0.0000214245831758299</v>
       </c>
     </row>
     <row r="127">
@@ -3853,16 +3847,16 @@
         <v>16</v>
       </c>
       <c r="E127" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F127" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G127" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H127" t="n">
-        <v>0.0217028851978872</v>
+        <v>0.0285509449840276</v>
       </c>
     </row>
     <row r="128">
@@ -3879,16 +3873,16 @@
         <v>17</v>
       </c>
       <c r="E128" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F128" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G128" t="n">
         <v>0</v>
       </c>
       <c r="H128" t="n">
-        <v>0.0525152748553331</v>
+        <v>0.0547081163064735</v>
       </c>
     </row>
     <row r="129">
@@ -3905,16 +3899,16 @@
         <v>11</v>
       </c>
       <c r="E129" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F129" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G129" t="n">
         <v>0</v>
       </c>
       <c r="H129" t="n">
-        <v>10.57110411056</v>
+        <v>10.6264746919281</v>
       </c>
     </row>
     <row r="130">
@@ -3931,16 +3925,16 @@
         <v>12</v>
       </c>
       <c r="E130" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F130" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G130" t="n">
         <v>0</v>
       </c>
       <c r="H130" t="n">
-        <v>11.3273604923011</v>
+        <v>8.2454291632263</v>
       </c>
     </row>
     <row r="131">
@@ -3957,16 +3951,16 @@
         <v>13</v>
       </c>
       <c r="E131" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F131" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G131" t="n">
         <v>0</v>
       </c>
       <c r="H131" t="n">
-        <v>41.9362536604355</v>
+        <v>45.3524079863932</v>
       </c>
     </row>
     <row r="132">
@@ -3983,7 +3977,7 @@
         <v>14</v>
       </c>
       <c r="E132" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F132" t="n">
         <v>0</v>
@@ -3992,7 +3986,7 @@
         <v>0</v>
       </c>
       <c r="H132" t="n">
-        <v>1997.98046501088</v>
+        <v>2085.98101428628</v>
       </c>
     </row>
     <row r="133">
@@ -4009,7 +4003,7 @@
         <v>15</v>
       </c>
       <c r="E133" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F133" t="n">
         <v>0</v>
@@ -4018,7 +4012,7 @@
         <v>0</v>
       </c>
       <c r="H133" t="n">
-        <v>2003.0764994734</v>
+        <v>1746.89206114818</v>
       </c>
     </row>
     <row r="134">
@@ -4035,16 +4029,16 @@
         <v>16</v>
       </c>
       <c r="E134" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F134" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G134" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H134" t="n">
-        <v>4.57067395805607</v>
+        <v>4.59227991637139</v>
       </c>
     </row>
     <row r="135">
@@ -4061,16 +4055,16 @@
         <v>11</v>
       </c>
       <c r="E135" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F135" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G135" t="n">
         <v>0</v>
       </c>
       <c r="H135" t="n">
-        <v>0.164835164835165</v>
+        <v>0.169230769230769</v>
       </c>
     </row>
     <row r="136">
@@ -4087,16 +4081,16 @@
         <v>12</v>
       </c>
       <c r="E136" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F136" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G136" t="n">
         <v>0</v>
       </c>
       <c r="H136" t="n">
-        <v>0.165289883395173</v>
+        <v>0.206612354243966</v>
       </c>
     </row>
     <row r="137">
@@ -4113,16 +4107,16 @@
         <v>13</v>
       </c>
       <c r="E137" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F137" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G137" t="n">
         <v>0</v>
       </c>
       <c r="H137" t="n">
-        <v>0.147904311263463</v>
+        <v>0.187639797871558</v>
       </c>
     </row>
     <row r="138">
@@ -4139,7 +4133,7 @@
         <v>14</v>
       </c>
       <c r="E138" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F138" t="n">
         <v>0</v>
@@ -4148,7 +4142,7 @@
         <v>0</v>
       </c>
       <c r="H138" t="n">
-        <v>0.169230769230769</v>
+        <v>0.147252747252747</v>
       </c>
     </row>
     <row r="139">
@@ -4165,16 +4159,16 @@
         <v>15</v>
       </c>
       <c r="E139" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F139" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G139" t="n">
         <v>0</v>
       </c>
       <c r="H139" t="n">
-        <v>0.173626373626374</v>
+        <v>0.138461538461538</v>
       </c>
     </row>
     <row r="140">
@@ -4191,16 +4185,16 @@
         <v>16</v>
       </c>
       <c r="E140" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F140" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G140" t="n">
         <v>5</v>
       </c>
       <c r="H140" t="n">
-        <v>0.389010989010989</v>
+        <v>0.362637362637363</v>
       </c>
     </row>
     <row r="141">
@@ -4217,16 +4211,16 @@
         <v>17</v>
       </c>
       <c r="E141" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F141" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G141" t="n">
         <v>0</v>
       </c>
       <c r="H141" t="n">
-        <v>0.0633615550466427</v>
+        <v>0.0501171383738601</v>
       </c>
     </row>
     <row r="142">
@@ -11796,30 +11790,30 @@
         <v>42</v>
       </c>
       <c r="G9" t="n">
-        <v>0.0482579570851503</v>
+        <v>0.0557705718084619</v>
       </c>
       <c r="H9" t="n">
-        <v>2.73981635833066</v>
+        <v>3.27225575941635</v>
       </c>
       <c r="I9" t="n">
-        <v>0.00716953725159897</v>
+        <v>0.0013376048203394</v>
       </c>
       <c r="J9" t="n">
-        <v>0.0466019921353933</v>
+        <v>0.0147136530237334</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="D10" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E10" t="n">
         <v>15</v>
@@ -11828,27 +11822,27 @@
         <v>43</v>
       </c>
       <c r="G10" t="n">
-        <v>0.0723979715730904</v>
+        <v>-85.6346636672553</v>
       </c>
       <c r="H10" t="n">
-        <v>3.74662757335061</v>
+        <v>-6.83593874560851</v>
       </c>
       <c r="I10" t="n">
-        <v>0.00028667480706331</v>
+        <v>0.0000119549092191627</v>
       </c>
       <c r="J10" t="n">
-        <v>0.00372677249182303</v>
+        <v>0.0227501922440666</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="B11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C11" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="D11" t="s">
         <v>16</v>
@@ -11857,179 +11851,179 @@
         <v>15</v>
       </c>
       <c r="F11" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.0838385746970638</v>
+        <v>74.8549263408796</v>
       </c>
       <c r="H11" t="n">
-        <v>-3.08472222924054</v>
+        <v>3.87359960945366</v>
       </c>
       <c r="I11" t="n">
-        <v>0.00238074741903707</v>
+        <v>0.00191974018964546</v>
       </c>
       <c r="J11" t="n">
-        <v>0.0309497164474819</v>
+        <v>0.0328140483750073</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="B12" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C12" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="D12" t="s">
         <v>16</v>
       </c>
       <c r="E12" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F12" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="G12" t="n">
-        <v>0.0629871851921108</v>
+        <v>52.3617052538158</v>
       </c>
       <c r="H12" t="n">
-        <v>2.92454809534197</v>
+        <v>3.61287502952434</v>
       </c>
       <c r="I12" t="n">
-        <v>0.00422159301284672</v>
+        <v>0.00315326346370199</v>
       </c>
       <c r="J12" t="n">
-        <v>0.0461054390039062</v>
+        <v>0.0355868305189225</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="B13" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C13" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="D13" t="s">
         <v>16</v>
       </c>
       <c r="E13" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F13" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.0607423709882282</v>
+        <v>105.220702137207</v>
       </c>
       <c r="H13" t="n">
-        <v>-2.88616046802902</v>
+        <v>4.11706595069739</v>
       </c>
       <c r="I13" t="n">
-        <v>0.00472876297475961</v>
+        <v>0.00121372633306425</v>
       </c>
       <c r="J13" t="n">
-        <v>0.0461054390039062</v>
+        <v>0.0328140483750073</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="B14" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C14" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="D14" t="s">
         <v>16</v>
       </c>
       <c r="E14" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F14" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="G14" t="n">
-        <v>0.06680919956309</v>
+        <v>70.7198983485343</v>
       </c>
       <c r="H14" t="n">
-        <v>3.22471887945743</v>
+        <v>3.62514795240969</v>
       </c>
       <c r="I14" t="n">
-        <v>0.00167806649596977</v>
+        <v>0.00308015029081166</v>
       </c>
       <c r="J14" t="n">
-        <v>0.0461054390039062</v>
+        <v>0.0355868305189225</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C15" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="D15" t="s">
         <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F15" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G15" t="n">
-        <v>0.0637034179289725</v>
+        <v>126.343212164399</v>
       </c>
       <c r="H15" t="n">
-        <v>3.02242842972628</v>
+        <v>3.83210180603845</v>
       </c>
       <c r="I15" t="n">
-        <v>0.0031463427025076</v>
+        <v>0.0020768385047473</v>
       </c>
       <c r="J15" t="n">
-        <v>0.0461054390039062</v>
+        <v>0.0328140483750073</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B16" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="C16" t="s">
         <v>18</v>
       </c>
       <c r="D16" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E16" t="n">
         <v>15</v>
       </c>
       <c r="F16" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="G16" t="n">
-        <v>-85.6346636672553</v>
+        <v>118.39415375599</v>
       </c>
       <c r="H16" t="n">
-        <v>-6.83593874560851</v>
+        <v>3.93690987073159</v>
       </c>
       <c r="I16" t="n">
-        <v>0.0000119549092191627</v>
+        <v>0.00170311441598215</v>
       </c>
       <c r="J16" t="n">
-        <v>0.0227501922440666</v>
+        <v>0.0328140483750073</v>
       </c>
     </row>
     <row r="17">
@@ -12049,16 +12043,16 @@
         <v>15</v>
       </c>
       <c r="F17" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="G17" t="n">
-        <v>74.8549263408796</v>
+        <v>52.5949371375936</v>
       </c>
       <c r="H17" t="n">
-        <v>3.87359960945366</v>
+        <v>4.14917428770798</v>
       </c>
       <c r="I17" t="n">
-        <v>0.00191974018964546</v>
+        <v>0.00114298519561347</v>
       </c>
       <c r="J17" t="n">
         <v>0.0328140483750073</v>
@@ -12066,7 +12060,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="B18" t="s">
         <v>21</v>
@@ -12081,19 +12075,19 @@
         <v>15</v>
       </c>
       <c r="F18" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="G18" t="n">
-        <v>52.3617052538158</v>
+        <v>9.95923094627214</v>
       </c>
       <c r="H18" t="n">
-        <v>3.61287502952434</v>
+        <v>4.03012047779369</v>
       </c>
       <c r="I18" t="n">
-        <v>0.00315326346370199</v>
+        <v>0.00142876685682359</v>
       </c>
       <c r="J18" t="n">
-        <v>0.0355868305189225</v>
+        <v>0.0157164354250594</v>
       </c>
     </row>
     <row r="19">
@@ -12101,7 +12095,7 @@
         <v>27</v>
       </c>
       <c r="B19" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C19" t="s">
         <v>18</v>
@@ -12110,86 +12104,86 @@
         <v>16</v>
       </c>
       <c r="E19" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F19" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="G19" t="n">
-        <v>105.220702137207</v>
+        <v>-156.142596682866</v>
       </c>
       <c r="H19" t="n">
-        <v>4.11706595069739</v>
+        <v>-4.62656942736316</v>
       </c>
       <c r="I19" t="n">
-        <v>0.00121372633306425</v>
+        <v>0.000583539829246223</v>
       </c>
       <c r="J19" t="n">
-        <v>0.0328140483750073</v>
+        <v>0.0460996465104516</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="B20" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="C20" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D20" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E20" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F20" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="G20" t="n">
-        <v>70.7198983485343</v>
+        <v>0.711455470357307</v>
       </c>
       <c r="H20" t="n">
-        <v>3.62514795240969</v>
+        <v>3.50710785038474</v>
       </c>
       <c r="I20" t="n">
-        <v>0.00308015029081166</v>
+        <v>0.00432487925868763</v>
       </c>
       <c r="J20" t="n">
-        <v>0.0355868305189225</v>
+        <v>0.0475736718455639</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B21" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="C21" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D21" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E21" t="n">
         <v>15</v>
       </c>
       <c r="F21" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="G21" t="n">
-        <v>126.343212164399</v>
+        <v>-0.874557588933838</v>
       </c>
       <c r="H21" t="n">
-        <v>3.83210180603845</v>
+        <v>-6.50262184884611</v>
       </c>
       <c r="I21" t="n">
-        <v>0.0020768385047473</v>
+        <v>0.0000199539861675725</v>
       </c>
       <c r="J21" t="n">
-        <v>0.0328140483750073</v>
+        <v>0.0379724356768904</v>
       </c>
     </row>
     <row r="22">
@@ -12200,7 +12194,7 @@
         <v>21</v>
       </c>
       <c r="C22" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D22" t="s">
         <v>16</v>
@@ -12209,19 +12203,19 @@
         <v>15</v>
       </c>
       <c r="F22" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G22" t="n">
-        <v>118.39415375599</v>
+        <v>0.746428571428571</v>
       </c>
       <c r="H22" t="n">
-        <v>3.93690987073159</v>
+        <v>4.04421614252928</v>
       </c>
       <c r="I22" t="n">
-        <v>0.00170311441598215</v>
+        <v>0.00139141108906305</v>
       </c>
       <c r="J22" t="n">
-        <v>0.0328140483750073</v>
+        <v>0.0379021155482388</v>
       </c>
     </row>
     <row r="23">
@@ -12232,7 +12226,7 @@
         <v>21</v>
       </c>
       <c r="C23" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D23" t="s">
         <v>16</v>
@@ -12241,30 +12235,30 @@
         <v>15</v>
       </c>
       <c r="F23" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="G23" t="n">
-        <v>52.5949371375936</v>
+        <v>0.735714285714286</v>
       </c>
       <c r="H23" t="n">
-        <v>4.14917428770798</v>
+        <v>3.91656106318704</v>
       </c>
       <c r="I23" t="n">
-        <v>0.00114298519561347</v>
+        <v>0.00176986864214427</v>
       </c>
       <c r="J23" t="n">
-        <v>0.0328140483750073</v>
+        <v>0.0379021155482388</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="B24" t="s">
         <v>21</v>
       </c>
       <c r="C24" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D24" t="s">
         <v>16</v>
@@ -12273,19 +12267,19 @@
         <v>15</v>
       </c>
       <c r="F24" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="G24" t="n">
-        <v>12.5378276194492</v>
+        <v>0.710714285714286</v>
       </c>
       <c r="H24" t="n">
-        <v>4.46268467753822</v>
+        <v>3.64262518878002</v>
       </c>
       <c r="I24" t="n">
-        <v>0.000639557128434251</v>
+        <v>0.00297899488680275</v>
       </c>
       <c r="J24" t="n">
-        <v>0.00831424266964527</v>
+        <v>0.0392234326762361</v>
       </c>
     </row>
     <row r="25">
@@ -12293,100 +12287,100 @@
         <v>27</v>
       </c>
       <c r="B25" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C25" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D25" t="s">
         <v>16</v>
       </c>
       <c r="E25" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F25" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="G25" t="n">
-        <v>-156.142596682866</v>
+        <v>0.75</v>
       </c>
       <c r="H25" t="n">
-        <v>-4.62656942736316</v>
+        <v>4.08831086321548</v>
       </c>
       <c r="I25" t="n">
-        <v>0.000583539829246223</v>
+        <v>0.00128089845093553</v>
       </c>
       <c r="J25" t="n">
-        <v>0.0460996465104516</v>
+        <v>0.0379021155482388</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="B26" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C26" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D26" t="s">
         <v>16</v>
       </c>
       <c r="E26" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F26" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="G26" t="n">
-        <v>12.1218730431815</v>
+        <v>0.725</v>
       </c>
       <c r="H26" t="n">
-        <v>4.24057394642642</v>
+        <v>3.79532338258449</v>
       </c>
       <c r="I26" t="n">
-        <v>0.00114629491254044</v>
+        <v>0.00222703231375421</v>
       </c>
       <c r="J26" t="n">
-        <v>0.0447055015890773</v>
+        <v>0.0379021155482388</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B27" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="C27" t="s">
         <v>19</v>
       </c>
       <c r="D27" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E27" t="n">
         <v>15</v>
       </c>
       <c r="F27" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="G27" t="n">
-        <v>-0.874557588933838</v>
+        <v>0.721428571428571</v>
       </c>
       <c r="H27" t="n">
-        <v>-6.50262184884611</v>
+        <v>3.75623041669329</v>
       </c>
       <c r="I27" t="n">
-        <v>0.0000199539861675725</v>
+        <v>0.00239886807267334</v>
       </c>
       <c r="J27" t="n">
-        <v>0.0379724356768904</v>
+        <v>0.0379021155482388</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="B28" t="s">
         <v>21</v>
@@ -12401,24 +12395,24 @@
         <v>15</v>
       </c>
       <c r="F28" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="G28" t="n">
-        <v>0.746428571428571</v>
+        <v>0.803571428571428</v>
       </c>
       <c r="H28" t="n">
-        <v>4.04421614252928</v>
+        <v>4.8677376148421</v>
       </c>
       <c r="I28" t="n">
-        <v>0.00139141108906305</v>
+        <v>0.000307265031812509</v>
       </c>
       <c r="J28" t="n">
-        <v>0.0379021155482388</v>
+        <v>0.0033799153499376</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B29" t="s">
         <v>21</v>
@@ -12433,24 +12427,24 @@
         <v>15</v>
       </c>
       <c r="F29" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="G29" t="n">
-        <v>0.735714285714286</v>
+        <v>-0.825</v>
       </c>
       <c r="H29" t="n">
-        <v>3.91656106318704</v>
+        <v>-5.26350652877657</v>
       </c>
       <c r="I29" t="n">
-        <v>0.00176986864214427</v>
+        <v>0.000153235570905647</v>
       </c>
       <c r="J29" t="n">
-        <v>0.0379021155482388</v>
+        <v>0.0486267545007253</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B30" t="s">
         <v>21</v>
@@ -12465,24 +12459,24 @@
         <v>15</v>
       </c>
       <c r="F30" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="G30" t="n">
-        <v>0.710714285714286</v>
+        <v>0.921428571428571</v>
       </c>
       <c r="H30" t="n">
-        <v>3.64262518878002</v>
+        <v>8.55044866398981</v>
       </c>
       <c r="I30" t="n">
-        <v>0.00297899488680275</v>
+        <v>0.00000107131729816209</v>
       </c>
       <c r="J30" t="n">
-        <v>0.0392234326762361</v>
+        <v>0.00194418108652679</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B31" t="s">
         <v>21</v>
@@ -12497,24 +12491,24 @@
         <v>15</v>
       </c>
       <c r="F31" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="G31" t="n">
-        <v>0.75</v>
+        <v>0.882142857142857</v>
       </c>
       <c r="H31" t="n">
-        <v>4.08831086321548</v>
+        <v>6.75314930887417</v>
       </c>
       <c r="I31" t="n">
-        <v>0.00128089845093553</v>
+        <v>0.0000135582106247888</v>
       </c>
       <c r="J31" t="n">
-        <v>0.0379021155482388</v>
+        <v>0.00645370825739945</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B32" t="s">
         <v>21</v>
@@ -12529,24 +12523,24 @@
         <v>15</v>
       </c>
       <c r="F32" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="G32" t="n">
-        <v>0.725</v>
+        <v>0.910714285714286</v>
       </c>
       <c r="H32" t="n">
-        <v>3.79532338258449</v>
+        <v>7.94996032435876</v>
       </c>
       <c r="I32" t="n">
-        <v>0.00222703231375421</v>
+        <v>0.00000239502083720704</v>
       </c>
       <c r="J32" t="n">
-        <v>0.0379021155482388</v>
+        <v>0.00194418108652679</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B33" t="s">
         <v>21</v>
@@ -12561,24 +12555,24 @@
         <v>15</v>
       </c>
       <c r="F33" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="G33" t="n">
-        <v>0.721428571428571</v>
+        <v>-0.871428571428571</v>
       </c>
       <c r="H33" t="n">
-        <v>3.75623041669329</v>
+        <v>-6.40537571094027</v>
       </c>
       <c r="I33" t="n">
-        <v>0.00239886807267334</v>
+        <v>0.0000232364778216326</v>
       </c>
       <c r="J33" t="n">
-        <v>0.0379021155482388</v>
+        <v>0.00884845075447769</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="B34" t="s">
         <v>21</v>
@@ -12593,27 +12587,27 @@
         <v>15</v>
       </c>
       <c r="F34" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="G34" t="n">
-        <v>0.875</v>
+        <v>0.907142857142857</v>
       </c>
       <c r="H34" t="n">
-        <v>6.51664535375884</v>
+        <v>7.77227377929872</v>
       </c>
       <c r="I34" t="n">
-        <v>0.0000195226138159411</v>
+        <v>0.00000306331053549389</v>
       </c>
       <c r="J34" t="n">
-        <v>0.000253793979607234</v>
+        <v>0.00194418108652679</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B35" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C35" t="s">
         <v>19</v>
@@ -12625,27 +12619,27 @@
         <v>15</v>
       </c>
       <c r="F35" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G35" t="n">
-        <v>-0.825</v>
+        <v>0.785714285714286</v>
       </c>
       <c r="H35" t="n">
-        <v>-5.26350652877657</v>
+        <v>4.57966519882549</v>
       </c>
       <c r="I35" t="n">
-        <v>0.000153235570905647</v>
+        <v>0.000516454747570588</v>
       </c>
       <c r="J35" t="n">
-        <v>0.0486267545007253</v>
+        <v>0.0407999250580765</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="B36" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C36" t="s">
         <v>19</v>
@@ -12657,27 +12651,27 @@
         <v>15</v>
       </c>
       <c r="F36" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G36" t="n">
-        <v>0.921428571428571</v>
+        <v>-0.6</v>
       </c>
       <c r="H36" t="n">
-        <v>8.55044866398981</v>
+        <v>-2.70416345659799</v>
       </c>
       <c r="I36" t="n">
-        <v>0.00000107131729816209</v>
+        <v>0.0180500879415</v>
       </c>
       <c r="J36" t="n">
-        <v>0.00194418108652679</v>
+        <v>0.049637741839125</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="B37" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C37" t="s">
         <v>19</v>
@@ -12689,27 +12683,27 @@
         <v>15</v>
       </c>
       <c r="F37" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G37" t="n">
-        <v>0.882142857142857</v>
+        <v>-0.607142857142857</v>
       </c>
       <c r="H37" t="n">
-        <v>6.75314930887417</v>
+        <v>-2.75497713055825</v>
       </c>
       <c r="I37" t="n">
-        <v>0.0000135582106247888</v>
+        <v>0.0163813067683071</v>
       </c>
       <c r="J37" t="n">
-        <v>0.00645370825739945</v>
+        <v>0.049637741839125</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="B38" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C38" t="s">
         <v>19</v>
@@ -12721,27 +12715,27 @@
         <v>15</v>
       </c>
       <c r="F38" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G38" t="n">
-        <v>0.910714285714286</v>
+        <v>0.735714285714286</v>
       </c>
       <c r="H38" t="n">
-        <v>7.94996032435876</v>
+        <v>3.91656106318704</v>
       </c>
       <c r="I38" t="n">
-        <v>0.00000239502083720704</v>
+        <v>0.00176986864214427</v>
       </c>
       <c r="J38" t="n">
-        <v>0.00194418108652679</v>
+        <v>0.019468555063587</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="B39" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C39" t="s">
         <v>19</v>
@@ -12753,19 +12747,19 @@
         <v>15</v>
       </c>
       <c r="F39" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G39" t="n">
-        <v>-0.871428571428571</v>
+        <v>-0.639285714285714</v>
       </c>
       <c r="H39" t="n">
-        <v>-6.40537571094027</v>
+        <v>-2.99748954833848</v>
       </c>
       <c r="I39" t="n">
-        <v>0.0000232364778216326</v>
+        <v>0.0102884466195942</v>
       </c>
       <c r="J39" t="n">
-        <v>0.00884845075447769</v>
+        <v>0.049637741839125</v>
       </c>
     </row>
     <row r="40">
@@ -12773,39 +12767,39 @@
         <v>28</v>
       </c>
       <c r="B40" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C40" t="s">
         <v>19</v>
       </c>
       <c r="D40" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E40" t="n">
         <v>15</v>
       </c>
       <c r="F40" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G40" t="n">
-        <v>0.907142857142857</v>
+        <v>0.875</v>
       </c>
       <c r="H40" t="n">
-        <v>7.77227377929872</v>
+        <v>6.51664535375884</v>
       </c>
       <c r="I40" t="n">
-        <v>0.00000306331053549389</v>
+        <v>0.0000195226138159411</v>
       </c>
       <c r="J40" t="n">
-        <v>0.00194418108652679</v>
+        <v>0.0371710567055519</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B41" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C41" t="s">
         <v>19</v>
@@ -12814,30 +12808,30 @@
         <v>16</v>
       </c>
       <c r="E41" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F41" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G41" t="n">
-        <v>0.785714285714286</v>
+        <v>0.912087912087912</v>
       </c>
       <c r="H41" t="n">
-        <v>4.57966519882549</v>
+        <v>7.70635653434765</v>
       </c>
       <c r="I41" t="n">
-        <v>0.000516454747570588</v>
+        <v>0.0000055020997463449</v>
       </c>
       <c r="J41" t="n">
-        <v>0.0407999250580765</v>
+        <v>0.0104759979170407</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="B42" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C42" t="s">
         <v>19</v>
@@ -12846,30 +12840,30 @@
         <v>16</v>
       </c>
       <c r="E42" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F42" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.682142857142857</v>
+        <v>-0.85054945054945</v>
       </c>
       <c r="H42" t="n">
-        <v>-3.36356315508022</v>
+        <v>-5.60261895086263</v>
       </c>
       <c r="I42" t="n">
-        <v>0.00508632646897726</v>
+        <v>0.00011565615890989</v>
       </c>
       <c r="J42" t="n">
-        <v>0.0330611220483522</v>
+        <v>0.0091368365538813</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="B43" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C43" t="s">
         <v>19</v>
@@ -12878,30 +12872,30 @@
         <v>16</v>
       </c>
       <c r="E43" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F43" t="s">
         <v>60</v>
       </c>
       <c r="G43" t="n">
-        <v>-0.628571428571428</v>
+        <v>0.815384615384615</v>
       </c>
       <c r="H43" t="n">
-        <v>-2.9139711855431</v>
+        <v>4.87904547486112</v>
       </c>
       <c r="I43" t="n">
-        <v>0.0120795391759058</v>
+        <v>0.000379132238200581</v>
       </c>
       <c r="J43" t="n">
-        <v>0.0392585023216937</v>
+        <v>0.0449271702267688</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="B44" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C44" t="s">
         <v>19</v>
@@ -12910,22 +12904,22 @@
         <v>16</v>
       </c>
       <c r="E44" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F44" t="s">
         <v>61</v>
       </c>
       <c r="G44" t="n">
-        <v>0.753571428571428</v>
+        <v>0.872527472527473</v>
       </c>
       <c r="H44" t="n">
-        <v>4.13322302468662</v>
+        <v>6.18653302499502</v>
       </c>
       <c r="I44" t="n">
-        <v>0.00117758302348883</v>
+        <v>0.0000468062120725075</v>
       </c>
       <c r="J44" t="n">
-        <v>0.0153085793053548</v>
+        <v>0.0110930722611843</v>
       </c>
     </row>
     <row r="45">
@@ -12933,7 +12927,7 @@
         <v>8</v>
       </c>
       <c r="B45" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C45" t="s">
         <v>19</v>
@@ -12942,62 +12936,62 @@
         <v>16</v>
       </c>
       <c r="E45" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F45" t="s">
         <v>62</v>
       </c>
       <c r="G45" t="n">
-        <v>0.628571428571428</v>
+        <v>0.793406593406593</v>
       </c>
       <c r="H45" t="n">
-        <v>2.9139711855431</v>
+        <v>4.5153229593002</v>
       </c>
       <c r="I45" t="n">
-        <v>0.0120795391759058</v>
+        <v>0.000707534135618204</v>
       </c>
       <c r="J45" t="n">
-        <v>0.0392585023216937</v>
+        <v>0.0176645525734471</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="B46" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C46" t="s">
         <v>19</v>
       </c>
       <c r="D46" t="s">
+        <v>16</v>
+      </c>
+      <c r="E46" t="n">
         <v>14</v>
-      </c>
-      <c r="E46" t="n">
-        <v>15</v>
       </c>
       <c r="F46" t="s">
         <v>63</v>
       </c>
       <c r="G46" t="n">
-        <v>0.875</v>
+        <v>-0.753846153846154</v>
       </c>
       <c r="H46" t="n">
-        <v>6.51664535375884</v>
+        <v>-3.97442481770368</v>
       </c>
       <c r="I46" t="n">
-        <v>0.0000195226138159411</v>
+        <v>0.00184472528925722</v>
       </c>
       <c r="J46" t="n">
-        <v>0.0371710567055519</v>
+        <v>0.0176645525734471</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="B47" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C47" t="s">
         <v>19</v>
@@ -13012,24 +13006,24 @@
         <v>64</v>
       </c>
       <c r="G47" t="n">
-        <v>0.912087912087912</v>
+        <v>-0.753846153846154</v>
       </c>
       <c r="H47" t="n">
-        <v>7.70635653434765</v>
+        <v>-3.97442481770368</v>
       </c>
       <c r="I47" t="n">
-        <v>0.0000055020997463449</v>
+        <v>0.00184472528925722</v>
       </c>
       <c r="J47" t="n">
-        <v>0.0104759979170407</v>
+        <v>0.0176645525734471</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="B48" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C48" t="s">
         <v>19</v>
@@ -13041,24 +13035,24 @@
         <v>14</v>
       </c>
       <c r="F48" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="G48" t="n">
-        <v>-0.85054945054945</v>
+        <v>0.745054945054945</v>
       </c>
       <c r="H48" t="n">
-        <v>-5.60261895086263</v>
+        <v>3.86946636014232</v>
       </c>
       <c r="I48" t="n">
-        <v>0.00011565615890989</v>
+        <v>0.00223003731674207</v>
       </c>
       <c r="J48" t="n">
-        <v>0.0091368365538813</v>
+        <v>0.0176645525734471</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="B49" t="s">
         <v>26</v>
@@ -13073,24 +13067,24 @@
         <v>14</v>
       </c>
       <c r="F49" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G49" t="n">
-        <v>0.815384615384615</v>
+        <v>-0.736263736263736</v>
       </c>
       <c r="H49" t="n">
-        <v>4.87904547486112</v>
+        <v>-3.76904446810218</v>
       </c>
       <c r="I49" t="n">
-        <v>0.000379132238200581</v>
+        <v>0.00267644735961319</v>
       </c>
       <c r="J49" t="n">
-        <v>0.0449271702267688</v>
+        <v>0.0176645525734471</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B50" t="s">
         <v>26</v>
@@ -13105,24 +13099,24 @@
         <v>14</v>
       </c>
       <c r="F50" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G50" t="n">
-        <v>0.872527472527473</v>
+        <v>0.92967032967033</v>
       </c>
       <c r="H50" t="n">
-        <v>6.18653302499502</v>
+        <v>8.74195855673915</v>
       </c>
       <c r="I50" t="n">
-        <v>0.0000468062120725075</v>
+        <v>0.00000149952507032915</v>
       </c>
       <c r="J50" t="n">
-        <v>0.0110930722611843</v>
+        <v>0.00856378767664976</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="B51" t="s">
         <v>26</v>
@@ -13137,24 +13131,24 @@
         <v>14</v>
       </c>
       <c r="F51" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="G51" t="n">
-        <v>0.876923076923077</v>
+        <v>0.89010989010989</v>
       </c>
       <c r="H51" t="n">
-        <v>6.3203418666616</v>
+        <v>6.76567946363491</v>
       </c>
       <c r="I51" t="n">
-        <v>0.0000382969810544994</v>
+        <v>0.0000199854042247814</v>
       </c>
       <c r="J51" t="n">
-        <v>0.00110756468719485</v>
+        <v>0.0285341608819316</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="B52" t="s">
         <v>26</v>
@@ -13169,24 +13163,24 @@
         <v>14</v>
       </c>
       <c r="F52" t="s">
-        <v>45</v>
+        <v>69</v>
       </c>
       <c r="G52" t="n">
-        <v>-0.868131868131868</v>
+        <v>0.898901098901099</v>
       </c>
       <c r="H52" t="n">
-        <v>-6.05902341189422</v>
+        <v>7.10686627911196</v>
       </c>
       <c r="I52" t="n">
-        <v>0.0000567981890869155</v>
+        <v>0.0000123587008656009</v>
       </c>
       <c r="J52" t="n">
-        <v>0.00110756468719485</v>
+        <v>0.0285341608819316</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="B53" t="s">
         <v>26</v>
@@ -13201,24 +13195,24 @@
         <v>14</v>
       </c>
       <c r="F53" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G53" t="n">
-        <v>-0.74945054945055</v>
+        <v>0.885714285714286</v>
       </c>
       <c r="H53" t="n">
-        <v>-3.92135393228648</v>
+        <v>6.60922220702392</v>
       </c>
       <c r="I53" t="n">
-        <v>0.00203014554910065</v>
+        <v>0.0000250400449891747</v>
       </c>
       <c r="J53" t="n">
-        <v>0.0197939191037313</v>
+        <v>0.0286007393866353</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="B54" t="s">
         <v>26</v>
@@ -13233,210 +13227,18 @@
         <v>14</v>
       </c>
       <c r="F54" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="G54" t="n">
-        <v>0.767032967032967</v>
+        <v>-0.894505494505494</v>
       </c>
       <c r="H54" t="n">
-        <v>4.14128474862473</v>
+        <v>-6.93123750597749</v>
       </c>
       <c r="I54" t="n">
-        <v>0.00136768238824561</v>
+        <v>0.0000157983084868006</v>
       </c>
       <c r="J54" t="n">
-        <v>0.0177798710471929</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="s">
-        <v>8</v>
-      </c>
-      <c r="B55" t="s">
-        <v>26</v>
-      </c>
-      <c r="C55" t="s">
-        <v>19</v>
-      </c>
-      <c r="D55" t="s">
-        <v>16</v>
-      </c>
-      <c r="E55" t="n">
-        <v>14</v>
-      </c>
-      <c r="F55" t="s">
-        <v>47</v>
-      </c>
-      <c r="G55" t="n">
-        <v>0.70989010989011</v>
-      </c>
-      <c r="H55" t="n">
-        <v>3.4915348503379</v>
-      </c>
-      <c r="I55" t="n">
-        <v>0.00445074141876422</v>
-      </c>
-      <c r="J55" t="n">
-        <v>0.034715783066361</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="s">
-        <v>28</v>
-      </c>
-      <c r="B56" t="s">
-        <v>26</v>
-      </c>
-      <c r="C56" t="s">
-        <v>19</v>
-      </c>
-      <c r="D56" t="s">
-        <v>16</v>
-      </c>
-      <c r="E56" t="n">
-        <v>14</v>
-      </c>
-      <c r="F56" t="s">
-        <v>69</v>
-      </c>
-      <c r="G56" t="n">
-        <v>0.92967032967033</v>
-      </c>
-      <c r="H56" t="n">
-        <v>8.74195855673915</v>
-      </c>
-      <c r="I56" t="n">
-        <v>0.00000149952507032915</v>
-      </c>
-      <c r="J56" t="n">
-        <v>0.00856378767664976</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="s">
-        <v>28</v>
-      </c>
-      <c r="B57" t="s">
-        <v>26</v>
-      </c>
-      <c r="C57" t="s">
-        <v>19</v>
-      </c>
-      <c r="D57" t="s">
-        <v>16</v>
-      </c>
-      <c r="E57" t="n">
-        <v>14</v>
-      </c>
-      <c r="F57" t="s">
-        <v>70</v>
-      </c>
-      <c r="G57" t="n">
-        <v>0.89010989010989</v>
-      </c>
-      <c r="H57" t="n">
-        <v>6.76567946363491</v>
-      </c>
-      <c r="I57" t="n">
-        <v>0.0000199854042247814</v>
-      </c>
-      <c r="J57" t="n">
-        <v>0.0285341608819316</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="s">
-        <v>28</v>
-      </c>
-      <c r="B58" t="s">
-        <v>26</v>
-      </c>
-      <c r="C58" t="s">
-        <v>19</v>
-      </c>
-      <c r="D58" t="s">
-        <v>16</v>
-      </c>
-      <c r="E58" t="n">
-        <v>14</v>
-      </c>
-      <c r="F58" t="s">
-        <v>71</v>
-      </c>
-      <c r="G58" t="n">
-        <v>0.898901098901099</v>
-      </c>
-      <c r="H58" t="n">
-        <v>7.10686627911196</v>
-      </c>
-      <c r="I58" t="n">
-        <v>0.0000123587008656009</v>
-      </c>
-      <c r="J58" t="n">
-        <v>0.0285341608819316</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="s">
-        <v>28</v>
-      </c>
-      <c r="B59" t="s">
-        <v>26</v>
-      </c>
-      <c r="C59" t="s">
-        <v>19</v>
-      </c>
-      <c r="D59" t="s">
-        <v>16</v>
-      </c>
-      <c r="E59" t="n">
-        <v>14</v>
-      </c>
-      <c r="F59" t="s">
-        <v>72</v>
-      </c>
-      <c r="G59" t="n">
-        <v>0.885714285714286</v>
-      </c>
-      <c r="H59" t="n">
-        <v>6.60922220702392</v>
-      </c>
-      <c r="I59" t="n">
-        <v>0.0000250400449891747</v>
-      </c>
-      <c r="J59" t="n">
-        <v>0.0286007393866353</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="s">
-        <v>28</v>
-      </c>
-      <c r="B60" t="s">
-        <v>26</v>
-      </c>
-      <c r="C60" t="s">
-        <v>19</v>
-      </c>
-      <c r="D60" t="s">
-        <v>16</v>
-      </c>
-      <c r="E60" t="n">
-        <v>14</v>
-      </c>
-      <c r="F60" t="s">
-        <v>73</v>
-      </c>
-      <c r="G60" t="n">
-        <v>-0.894505494505494</v>
-      </c>
-      <c r="H60" t="n">
-        <v>-6.93123750597749</v>
-      </c>
-      <c r="I60" t="n">
-        <v>0.0000157983084868006</v>
-      </c>
-      <c r="J60" t="n">
         <v>0.0285341608819316</v>
       </c>
     </row>

</xml_diff>